<commit_message>
Add verified recipient emails for 4 North Wales / border leads
Snowdonia Cheese, Wild Horse Brewing, Different Dog and Hilltop Honey now have
confirmed contact addresses; Gmail drafts, tracker and brief updated to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EAcEcxgaTrHynQWoQanPC4
</commit_message>
<xml_diff>
--- a/outreach/vedri-outreach-tracker.xlsx
+++ b/outreach/vedri-outreach-tracker.xlsx
@@ -68,12 +68,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -114,13 +114,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -667,10 +667,14 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn / site contact form</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr"/>
+          <t>info@snowdonia-cheese.co.uk</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>info@snowdonia-cheese.co.uk</t>
+        </is>
+      </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Black Bomber deserves more than a product shot</t>
@@ -678,7 +682,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>Yes – add recipient</t>
+          <t>YES – ready to send</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
@@ -686,86 +690,94 @@
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr"/>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>Verified email – send-ready</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Wild Horse Brewing Co</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Drink — craft beer</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Llandudno, Conwy</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>North Wales ⭐</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>~7.5k IG / ~1,287 posts; lots of effort, little reach; design-led cans unused</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>DBW/Welsh Gov funding; capacity doubled 175k→350k L; new taproom</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>wildhorsebrewing.co.uk</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>@wildhorsebeer</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>~7.5k</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Dave &amp; Emma Faragher</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>LinkedIn / site contact form</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>sales@wildhorsebrewing.co.uk</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>sales@wildhorsebrewing.co.uk</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Those cans are wasted as thumbnails</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Yes – add recipient</t>
-        </is>
-      </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>YES – ready to send</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q6" s="5" t="inlineStr">
-        <is>
-          <t>Warmest travel pitch – on the doorstep</t>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>Verified email; warmest travel pitch – on the doorstep</t>
         </is>
       </c>
     </row>
@@ -825,10 +837,14 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn / site contact form</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr"/>
+          <t>feedme@differentdog.com</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>feedme@differentdog.com</t>
+        </is>
+      </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
           <t>£10m in, and the dogs aren't on camera enough</t>
@@ -836,7 +852,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>Yes – add recipient</t>
+          <t>YES – ready to send</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
@@ -846,167 +862,175 @@
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>~1 hr from DocShed</t>
+          <t>Verified email; ~1 hr from DocShed</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Hilltop Honey</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Food — honey</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Newtown, Powys</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Mid Wales</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>~39k IG / ~1,524 posts; jar photography heavy; lags commercial scale</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>£10m Santander (2024); sales £20m→£33m, target £50m; B-Corp; major multiples</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>hilltophoney.co.uk</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>@hilltop_honey</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>~39k</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Scott Davies (CEO)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>LinkedIn / site contact form</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>info@lovehilltop.com</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>info@lovehilltop.com</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>£33m in sales, 39k followers — the maths is off</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Yes – add recipient</t>
-        </is>
-      </c>
-      <c r="P8" s="5" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>YES – ready to send</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q8" s="5" t="inlineStr"/>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>Verified email</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Hip Pop</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Drink — gut soda</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Altrincham, Gtr Manchester</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>North West</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>~29k IG; invests in content but underweight vs US peers (millions)</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>~£7m raised (LadBible founders, ex-Olipop CFO); Waitrose &amp; Booths</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>drinkhippop.com</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>@drink.hip.pop</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>~29k</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Emma Thackray &amp; Kenny Goodman</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>hello@drinkhippop.com</t>
         </is>
       </c>
-      <c r="M9" s="6" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>hello@drinkhippop.com</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>29k is underweight for where Hip Pop's headed</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>YES – ready to send</t>
         </is>
       </c>
-      <c r="P9" s="6" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q9" s="6" t="inlineStr">
+      <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>Verified email – send-ready</t>
         </is>
@@ -1094,247 +1118,247 @@
       </c>
     </row>
     <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Adamo Foods</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Foodtech — mycelium steak</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>National</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>~995 IG followers / ~19 posts; near-absent owned audience</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>~£2m seed + €10m EU Horizon grant; consumer launch ~2027 (build-hype angle)</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>adamofoods.com</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>@adamo.foods</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>~995</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>Pierre Dupuis (CEO)</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>LinkedIn; UNVERIFIED contact@/marketing@adamofoods.com</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr"/>
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>€10m raised, 995 followers — that gap is the opportunity</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>Yes – add recipient</t>
         </is>
       </c>
-      <c r="P11" s="4" t="inlineStr">
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q11" s="4" t="inlineStr">
+      <c r="Q11" s="6" t="inlineStr">
         <is>
           <t>Highest-contrast story; verify email first</t>
         </is>
       </c>
     </row>
     <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>PURIFIED</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Footwear</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>National</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>~3.4k IG; world-first plastic-free shoe + royal exposure, static feed</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Prince William wore them at Earthshot 2024; raising investment</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>purified.eco</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>@purifiedfootwear</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>~3.4k</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Will Verona (founder)</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>enquiries@purified.eco (press: charlie@purified.eco)</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>enquiries@purified.eco</t>
         </is>
       </c>
-      <c r="N12" s="6" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>Prince William wore your shoes — where's the video?</t>
         </is>
       </c>
-      <c r="O12" s="6" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>YES – ready to send</t>
         </is>
       </c>
-      <c r="P12" s="6" t="inlineStr">
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q12" s="6" t="inlineStr">
+      <c r="Q12" s="4" t="inlineStr">
         <is>
           <t>Verified email – send-ready</t>
         </is>
       </c>
     </row>
     <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>ReBorn Homewares</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Homeware</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Wiltshire</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>National</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>~6.4k IG; styled static photography, no video engine</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Holly Branson + Conduit EIS backing; ~$550k angel (2025); John Lewis</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>reborn.homes</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>@reborn_homes</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>~6.4k</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Brian Walmsley (CEO)</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>LinkedIn (in/brianwalmsley) / site form</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr"/>
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>Waste into homeware — that's a film, not a photo</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>Yes – add recipient</t>
         </is>
       </c>
-      <c r="P13" s="4" t="inlineStr">
+      <c r="P13" s="6" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr">
+      <c r="Q13" s="6" t="inlineStr">
         <is>
           <t>Waste-to-product = ready-made video</t>
         </is>

</xml_diff>

<commit_message>
All 10 leads now have verified recipients; note vedri.studio send-as
Adds confirmed addresses for Forest Distillery, Adamo Foods, ReBorn Homewares
and ACTIPH Water. Documents that outreach should be sent from info@vedri.studio
via a Send mail as alias. Tracker and brief updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EAcEcxgaTrHynQWoQanPC4
</commit_message>
<xml_diff>
--- a/outreach/vedri-outreach-tracker.xlsx
+++ b/outreach/vedri-outreach-tracker.xlsx
@@ -49,7 +49,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -64,16 +64,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF4CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -115,12 +105,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -520,7 +504,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Legend:  Green rows = verified email, send-ready.  All other drafts are saved in Gmail with your own address as a placeholder — replace the To before sending.  Follower counts are search-surfaced (Aug 2026) — confirm on the live feed before quoting in line one.  Fill in the 'Reply status' and 'Notes' columns as you work through.</t>
+          <t>Legend:  All 10 drafts are saved in Gmail with confirmed recipients — send-ready.  Send FROM info@vedri.studio: add it as a verified 'Send mail as' alias, then pick it as the From address before sending.  Follower counts are search-surfaced (Aug 2026) — confirm on the live feed before quoting in line one.  Fill in the 'Reply status' and 'Notes' columns as you work through.</t>
         </is>
       </c>
     </row>
@@ -1037,164 +1021,172 @@
       </c>
     </row>
     <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>The Forest Distillery (Forest Gin)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Drink — spirits</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Macclesfield, Cheshire</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>North West</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>~16k IG; premium, cinematic product with almost no organic video</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Double double-gold SFWSC; 'World's Best 50 Gins'; Harvey Nichols</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>theforestdistillery.com</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>@forest_distillery</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>~16k</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Karl &amp; Lindsay Bond</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>LinkedIn / site contact form</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>team@theforestdistillery.com</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>team@theforestdistillery.com</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>The most beautiful bottle in Britain, hiding at 16k</t>
         </is>
       </c>
-      <c r="O10" s="5" t="inlineStr">
-        <is>
-          <t>Yes – add recipient</t>
-        </is>
-      </c>
-      <c r="P10" s="5" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>YES – ready to send</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q10" s="5" t="inlineStr">
-        <is>
-          <t>Most visually stunning product on the list</t>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Verified email; most visually stunning product on the list</t>
         </is>
       </c>
     </row>
     <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Adamo Foods</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Foodtech — mycelium steak</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>National</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>~995 IG followers / ~19 posts; near-absent owned audience</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>~£2m seed + €10m EU Horizon grant; consumer launch ~2027 (build-hype angle)</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>adamofoods.com</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>@adamo.foods</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>~995</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Pierre Dupuis (CEO)</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn; UNVERIFIED contact@/marketing@adamofoods.com</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr"/>
-      <c r="N11" s="6" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>contact@adamofoods.com</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>contact@adamofoods.com</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>€10m raised, 995 followers — that gap is the opportunity</t>
         </is>
       </c>
-      <c r="O11" s="6" t="inlineStr">
-        <is>
-          <t>Yes – add recipient</t>
-        </is>
-      </c>
-      <c r="P11" s="6" t="inlineStr">
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>YES – ready to send</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q11" s="6" t="inlineStr">
-        <is>
-          <t>Highest-contrast story; verify email first</t>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>Verified email; highest-contrast story</t>
         </is>
       </c>
     </row>
@@ -1284,162 +1276,174 @@
       </c>
     </row>
     <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>ReBorn Homewares</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Homeware</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Wiltshire</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>National</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>~6.4k IG; styled static photography, no video engine</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Holly Branson + Conduit EIS backing; ~$550k angel (2025); John Lewis</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>reborn.homes</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>@reborn_homes</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>~6.4k</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Brian Walmsley (CEO)</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn (in/brianwalmsley) / site form</t>
-        </is>
-      </c>
-      <c r="M13" s="6" t="inlineStr"/>
-      <c r="N13" s="6" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>support@reborn.homes</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>support@reborn.homes</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Waste into homeware — that's a film, not a photo</t>
         </is>
       </c>
-      <c r="O13" s="6" t="inlineStr">
-        <is>
-          <t>Yes – add recipient</t>
-        </is>
-      </c>
-      <c r="P13" s="6" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>YES – ready to send</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q13" s="6" t="inlineStr">
-        <is>
-          <t>Waste-to-product = ready-made video</t>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>Verified email; waste-to-product = ready-made video</t>
         </is>
       </c>
     </row>
     <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>ACTIPH Water</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Drink — water</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>National</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>IG ~26k but TikTok ~1,750 — dormant on the key beverage channel</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>~£10m+ raised; Tesco/Sainsbury's/Ocado/H&amp;B/BP; exports ~20 countries</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>actiphwater.com</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>@actiphwater</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>TikTok ~1,750</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Barnaby Hughes (CMO) / Jamie Douglas-Hamilton</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr">
-        <is>
-          <t>Barnaby: likely firstname@actiphwater.com (verify)</t>
-        </is>
-      </c>
-      <c r="M14" s="5" t="inlineStr"/>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>hello@actiphwater.com</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>hello@actiphwater.com</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Your TikTok's asleep — and it's costing you</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>Yes – add recipient</t>
-        </is>
-      </c>
-      <c r="P14" s="5" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>YES – ready to send</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>Not sent</t>
         </is>
       </c>
-      <c r="Q14" s="5" t="inlineStr"/>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>Verified email (general inbox)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Log 10 scheduled sends: CRM rows + tracker status
Adds crm-rows.tsv (paste-ready rows in the client CRM column order) and marks
all 10 leads as Scheduled 01-08-26 in the tracker.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EAcEcxgaTrHynQWoQanPC4
</commit_message>
<xml_diff>
--- a/outreach/vedri-outreach-tracker.xlsx
+++ b/outreach/vedri-outreach-tracker.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q5" s="4" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q6" s="4" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q7" s="4" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q8" s="4" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q9" s="4" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q10" s="4" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q12" s="4" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Scheduled 01-08-26</t>
         </is>
       </c>
       <c r="Q14" s="4" t="inlineStr">

</xml_diff>